<commit_message>
Copy trading app code fixed rel 1
</commit_message>
<xml_diff>
--- a/c-t-backend/conf/users.xlsx
+++ b/c-t-backend/conf/users.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20373"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBF01668-2316-46D1-8AD8-DABA5CAFDB26}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8357F131-B49C-48D1-B882-A97E8D389A0B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
   <si>
     <t>apiKey</t>
   </si>
@@ -40,30 +40,6 @@
     <t>quantity</t>
   </si>
   <si>
-    <t>abc123</t>
-  </si>
-  <si>
-    <t>pass123</t>
-  </si>
-  <si>
-    <t>REQ001</t>
-  </si>
-  <si>
-    <t>U1001</t>
-  </si>
-  <si>
-    <t>def456</t>
-  </si>
-  <si>
-    <t>pass456</t>
-  </si>
-  <si>
-    <t>REQ002</t>
-  </si>
-  <si>
-    <t>U1002</t>
-  </si>
-  <si>
     <t>ghi789</t>
   </si>
   <si>
@@ -98,6 +74,18 @@
   </si>
   <si>
     <t>U1005</t>
+  </si>
+  <si>
+    <t>04FCaiaW37pOKA</t>
+  </si>
+  <si>
+    <t>6LWnI8#Vl%nAsl*w</t>
+  </si>
+  <si>
+    <t>633639c53bf429be</t>
+  </si>
+  <si>
+    <t>313462c922c9bbf5</t>
   </si>
 </sst>
 </file>
@@ -418,7 +406,10 @@
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -443,16 +434,16 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" t="s">
-        <v>9</v>
+        <v>21</v>
+      </c>
+      <c r="D2">
+        <v>45937331</v>
       </c>
       <c r="E2" t="b">
         <v>1</v>
@@ -463,36 +454,36 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3">
+        <v>45937331</v>
+      </c>
+      <c r="E3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F3">
         <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" t="b">
-        <v>1</v>
-      </c>
-      <c r="F3">
-        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -503,19 +494,19 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D5" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="E5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5">
         <v>25</v>
@@ -523,19 +514,19 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B6" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="C6" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D6" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="E6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6">
         <v>30</v>

</xml_diff>